<commit_message>
chore(data): add 2026-2 data files ('26.07.10+)
</commit_message>
<xml_diff>
--- a/data/2026년 2학기 정규 시간표.xlsx
+++ b/data/2026년 2학기 정규 시간표.xlsx
@@ -22892,7 +22892,11 @@
         </is>
       </c>
       <c r="M383" t="inlineStr"/>
-      <c r="N383" t="inlineStr"/>
+      <c r="N383" t="inlineStr">
+        <is>
+          <t>(팀티칭)</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -22952,7 +22956,11 @@
         </is>
       </c>
       <c r="M384" t="inlineStr"/>
-      <c r="N384" t="inlineStr"/>
+      <c r="N384" t="inlineStr">
+        <is>
+          <t>(팀티칭)</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -52560,8 +52568,16 @@
           <t>김나미</t>
         </is>
       </c>
-      <c r="J873" t="inlineStr"/>
-      <c r="K873" t="inlineStr"/>
+      <c r="J873" t="inlineStr">
+        <is>
+          <t>금1~2</t>
+        </is>
+      </c>
+      <c r="K873" t="inlineStr">
+        <is>
+          <t>에스라관209호강의실(교직과목)(첨단강의실)</t>
+        </is>
+      </c>
       <c r="L873" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -52611,9 +52627,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I874" t="inlineStr"/>
-      <c r="J874" t="inlineStr"/>
-      <c r="K874" t="inlineStr"/>
+      <c r="I874" t="inlineStr">
+        <is>
+          <t>이재균</t>
+        </is>
+      </c>
+      <c r="J874" t="inlineStr">
+        <is>
+          <t>금5~6</t>
+        </is>
+      </c>
+      <c r="K874" t="inlineStr">
+        <is>
+          <t>에스라관209호강의실(교직과목)(첨단강의실)</t>
+        </is>
+      </c>
       <c r="L874" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -52667,9 +52695,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I875" t="inlineStr"/>
-      <c r="J875" t="inlineStr"/>
-      <c r="K875" t="inlineStr"/>
+      <c r="I875" t="inlineStr">
+        <is>
+          <t>문종주</t>
+        </is>
+      </c>
+      <c r="J875" t="inlineStr">
+        <is>
+          <t>월2~3</t>
+        </is>
+      </c>
+      <c r="K875" t="inlineStr">
+        <is>
+          <t>체육관203호(주경기장)</t>
+        </is>
+      </c>
       <c r="L875" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -52719,9 +52759,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I876" t="inlineStr"/>
-      <c r="J876" t="inlineStr"/>
-      <c r="K876" t="inlineStr"/>
+      <c r="I876" t="inlineStr">
+        <is>
+          <t>최순남</t>
+        </is>
+      </c>
+      <c r="J876" t="inlineStr">
+        <is>
+          <t>목1~2</t>
+        </is>
+      </c>
+      <c r="K876" t="inlineStr">
+        <is>
+          <t>에스라관209호강의실(교직과목)(첨단강의실)</t>
+        </is>
+      </c>
       <c r="L876" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -52775,9 +52827,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I877" t="inlineStr"/>
-      <c r="J877" t="inlineStr"/>
-      <c r="K877" t="inlineStr"/>
+      <c r="I877" t="inlineStr">
+        <is>
+          <t>이금선</t>
+        </is>
+      </c>
+      <c r="J877" t="inlineStr">
+        <is>
+          <t>수7~8</t>
+        </is>
+      </c>
+      <c r="K877" t="inlineStr">
+        <is>
+          <t>온라인(가상공간)</t>
+        </is>
+      </c>
       <c r="L877" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -52831,9 +52895,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I878" t="inlineStr"/>
-      <c r="J878" t="inlineStr"/>
-      <c r="K878" t="inlineStr"/>
+      <c r="I878" t="inlineStr">
+        <is>
+          <t>임지헌</t>
+        </is>
+      </c>
+      <c r="J878" t="inlineStr">
+        <is>
+          <t>금5~6</t>
+        </is>
+      </c>
+      <c r="K878" t="inlineStr">
+        <is>
+          <t>체육관203호(주경기장)</t>
+        </is>
+      </c>
       <c r="L878" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -52887,9 +52963,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I879" t="inlineStr"/>
-      <c r="J879" t="inlineStr"/>
-      <c r="K879" t="inlineStr"/>
+      <c r="I879" t="inlineStr">
+        <is>
+          <t>서경현</t>
+        </is>
+      </c>
+      <c r="J879" t="inlineStr">
+        <is>
+          <t>수5~6</t>
+        </is>
+      </c>
+      <c r="K879" t="inlineStr">
+        <is>
+          <t>에스라관306호강의실</t>
+        </is>
+      </c>
       <c r="L879" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -52943,9 +53031,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I880" t="inlineStr"/>
-      <c r="J880" t="inlineStr"/>
-      <c r="K880" t="inlineStr"/>
+      <c r="I880" t="inlineStr">
+        <is>
+          <t>유재홍</t>
+        </is>
+      </c>
+      <c r="J880" t="inlineStr">
+        <is>
+          <t>목3~4</t>
+        </is>
+      </c>
+      <c r="K880" t="inlineStr">
+        <is>
+          <t>체육관203호(주경기장)</t>
+        </is>
+      </c>
       <c r="L880" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -52999,9 +53099,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I881" t="inlineStr"/>
-      <c r="J881" t="inlineStr"/>
-      <c r="K881" t="inlineStr"/>
+      <c r="I881" t="inlineStr">
+        <is>
+          <t>이재구</t>
+        </is>
+      </c>
+      <c r="J881" t="inlineStr">
+        <is>
+          <t>화5~6</t>
+        </is>
+      </c>
+      <c r="K881" t="inlineStr">
+        <is>
+          <t>체육관203호(주경기장)</t>
+        </is>
+      </c>
       <c r="L881" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -53055,9 +53167,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I882" t="inlineStr"/>
-      <c r="J882" t="inlineStr"/>
-      <c r="K882" t="inlineStr"/>
+      <c r="I882" t="inlineStr">
+        <is>
+          <t>방은혜</t>
+        </is>
+      </c>
+      <c r="J882" t="inlineStr">
+        <is>
+          <t>화3~4</t>
+        </is>
+      </c>
+      <c r="K882" t="inlineStr">
+        <is>
+          <t>체육관203호(주경기장)</t>
+        </is>
+      </c>
       <c r="L882" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -53111,9 +53235,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I883" t="inlineStr"/>
-      <c r="J883" t="inlineStr"/>
-      <c r="K883" t="inlineStr"/>
+      <c r="I883" t="inlineStr">
+        <is>
+          <t>한승대</t>
+        </is>
+      </c>
+      <c r="J883" t="inlineStr">
+        <is>
+          <t>월2~3</t>
+        </is>
+      </c>
+      <c r="K883" t="inlineStr">
+        <is>
+          <t>바울관203호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L883" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -53167,9 +53303,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I884" t="inlineStr"/>
-      <c r="J884" t="inlineStr"/>
-      <c r="K884" t="inlineStr"/>
+      <c r="I884" t="inlineStr">
+        <is>
+          <t>문종주</t>
+        </is>
+      </c>
+      <c r="J884" t="inlineStr">
+        <is>
+          <t>월5~6</t>
+        </is>
+      </c>
+      <c r="K884" t="inlineStr">
+        <is>
+          <t>체육관102호(수영장)</t>
+        </is>
+      </c>
       <c r="L884" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -53223,7 +53371,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I885" t="inlineStr"/>
+      <c r="I885" t="inlineStr">
+        <is>
+          <t>구본학</t>
+        </is>
+      </c>
       <c r="J885" t="inlineStr"/>
       <c r="K885" t="inlineStr"/>
       <c r="L885" t="inlineStr">
@@ -53279,9 +53431,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I886" t="inlineStr"/>
-      <c r="J886" t="inlineStr"/>
-      <c r="K886" t="inlineStr"/>
+      <c r="I886" t="inlineStr">
+        <is>
+          <t>김수연</t>
+        </is>
+      </c>
+      <c r="J886" t="inlineStr">
+        <is>
+          <t>금3~4</t>
+        </is>
+      </c>
+      <c r="K886" t="inlineStr">
+        <is>
+          <t>다니엘관302호(中)강의실</t>
+        </is>
+      </c>
       <c r="L886" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -53335,9 +53499,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I887" t="inlineStr"/>
-      <c r="J887" t="inlineStr"/>
-      <c r="K887" t="inlineStr"/>
+      <c r="I887" t="inlineStr">
+        <is>
+          <t>김영미</t>
+        </is>
+      </c>
+      <c r="J887" t="inlineStr">
+        <is>
+          <t>금5~6</t>
+        </is>
+      </c>
+      <c r="K887" t="inlineStr">
+        <is>
+          <t>체육관 206호(스쿼시장)</t>
+        </is>
+      </c>
       <c r="L887" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -53391,9 +53567,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I888" t="inlineStr"/>
-      <c r="J888" t="inlineStr"/>
-      <c r="K888" t="inlineStr"/>
+      <c r="I888" t="inlineStr">
+        <is>
+          <t>박형길</t>
+        </is>
+      </c>
+      <c r="J888" t="inlineStr">
+        <is>
+          <t>화10~11</t>
+        </is>
+      </c>
+      <c r="K888" t="inlineStr">
+        <is>
+          <t>미지정</t>
+        </is>
+      </c>
       <c r="L888" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -53447,9 +53635,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I889" t="inlineStr"/>
-      <c r="J889" t="inlineStr"/>
-      <c r="K889" t="inlineStr"/>
+      <c r="I889" t="inlineStr">
+        <is>
+          <t>취업정보</t>
+        </is>
+      </c>
+      <c r="J889" t="inlineStr">
+        <is>
+          <t>월5~6</t>
+        </is>
+      </c>
+      <c r="K889" t="inlineStr">
+        <is>
+          <t>요한관221호(中)(교필토익전용)강의실</t>
+        </is>
+      </c>
       <c r="L889" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -53503,9 +53703,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I890" t="inlineStr"/>
-      <c r="J890" t="inlineStr"/>
-      <c r="K890" t="inlineStr"/>
+      <c r="I890" t="inlineStr">
+        <is>
+          <t>취업정보</t>
+        </is>
+      </c>
+      <c r="J890" t="inlineStr">
+        <is>
+          <t>월7~8</t>
+        </is>
+      </c>
+      <c r="K890" t="inlineStr">
+        <is>
+          <t>요한관221호(中)(교필토익전용)강의실</t>
+        </is>
+      </c>
       <c r="L890" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -53559,9 +53771,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I891" t="inlineStr"/>
-      <c r="J891" t="inlineStr"/>
-      <c r="K891" t="inlineStr"/>
+      <c r="I891" t="inlineStr">
+        <is>
+          <t>홍선미</t>
+        </is>
+      </c>
+      <c r="J891" t="inlineStr">
+        <is>
+          <t>목6~7</t>
+        </is>
+      </c>
+      <c r="K891" t="inlineStr">
+        <is>
+          <t>디자인관B108호(신체표현실)</t>
+        </is>
+      </c>
       <c r="L891" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -53615,9 +53839,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I892" t="inlineStr"/>
-      <c r="J892" t="inlineStr"/>
-      <c r="K892" t="inlineStr"/>
+      <c r="I892" t="inlineStr">
+        <is>
+          <t>이재구</t>
+        </is>
+      </c>
+      <c r="J892" t="inlineStr">
+        <is>
+          <t>화7~8</t>
+        </is>
+      </c>
+      <c r="K892" t="inlineStr">
+        <is>
+          <t>다니엘관406호(PBL 전용 Lab. 中)강의실</t>
+        </is>
+      </c>
       <c r="L892" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -54227,9 +54463,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I903" t="inlineStr"/>
-      <c r="J903" t="inlineStr"/>
-      <c r="K903" t="inlineStr"/>
+      <c r="I903" t="inlineStr">
+        <is>
+          <t>심성용</t>
+        </is>
+      </c>
+      <c r="J903" t="inlineStr">
+        <is>
+          <t>목3~4</t>
+        </is>
+      </c>
+      <c r="K903" t="inlineStr">
+        <is>
+          <t>에스라관209호강의실(교직과목)(첨단강의실)</t>
+        </is>
+      </c>
       <c r="L903" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -54279,9 +54527,21 @@
           <t>2</t>
         </is>
       </c>
-      <c r="I904" t="inlineStr"/>
-      <c r="J904" t="inlineStr"/>
-      <c r="K904" t="inlineStr"/>
+      <c r="I904" t="inlineStr">
+        <is>
+          <t>김나미</t>
+        </is>
+      </c>
+      <c r="J904" t="inlineStr">
+        <is>
+          <t>금3~4</t>
+        </is>
+      </c>
+      <c r="K904" t="inlineStr">
+        <is>
+          <t>에스라관209호강의실(교직과목)(첨단강의실)</t>
+        </is>
+      </c>
       <c r="L904" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -56151,7 +56411,7 @@
       </c>
       <c r="K933" t="inlineStr">
         <is>
-          <t>에스라관209호강의실(교직과목)(첨단강의실)</t>
+          <t>사무엘관210호(PBL소형)강의실</t>
         </is>
       </c>
       <c r="L933" t="inlineStr">
@@ -56339,9 +56599,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I936" t="inlineStr"/>
-      <c r="J936" t="inlineStr"/>
-      <c r="K936" t="inlineStr"/>
+      <c r="I936" t="inlineStr">
+        <is>
+          <t>Lee Jeeny Jeeyoun</t>
+        </is>
+      </c>
+      <c r="J936" t="inlineStr">
+        <is>
+          <t>수6~8</t>
+        </is>
+      </c>
+      <c r="K936" t="inlineStr">
+        <is>
+          <t>에스라관209호강의실(교직과목)(첨단강의실)</t>
+        </is>
+      </c>
       <c r="L936" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -56395,9 +56667,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I937" t="inlineStr"/>
-      <c r="J937" t="inlineStr"/>
-      <c r="K937" t="inlineStr"/>
+      <c r="I937" t="inlineStr">
+        <is>
+          <t>김명희</t>
+        </is>
+      </c>
+      <c r="J937" t="inlineStr">
+        <is>
+          <t>월4~6</t>
+        </is>
+      </c>
+      <c r="K937" t="inlineStr">
+        <is>
+          <t>다니엘관402호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L937" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -56452,8 +56736,16 @@
         </is>
       </c>
       <c r="I938" t="inlineStr"/>
-      <c r="J938" t="inlineStr"/>
-      <c r="K938" t="inlineStr"/>
+      <c r="J938" t="inlineStr">
+        <is>
+          <t>월4~6</t>
+        </is>
+      </c>
+      <c r="K938" t="inlineStr">
+        <is>
+          <t>바울관203호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L938" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -58971,9 +59263,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I983" t="inlineStr"/>
-      <c r="J983" t="inlineStr"/>
-      <c r="K983" t="inlineStr"/>
+      <c r="I983" t="inlineStr">
+        <is>
+          <t>이병희</t>
+        </is>
+      </c>
+      <c r="J983" t="inlineStr">
+        <is>
+          <t>금5~7</t>
+        </is>
+      </c>
+      <c r="K983" t="inlineStr">
+        <is>
+          <t>다니엘관302호(中)강의실</t>
+        </is>
+      </c>
       <c r="L983" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -59027,9 +59331,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I984" t="inlineStr"/>
-      <c r="J984" t="inlineStr"/>
-      <c r="K984" t="inlineStr"/>
+      <c r="I984" t="inlineStr">
+        <is>
+          <t>김나미</t>
+        </is>
+      </c>
+      <c r="J984" t="inlineStr">
+        <is>
+          <t>목7~9</t>
+        </is>
+      </c>
+      <c r="K984" t="inlineStr">
+        <is>
+          <t>다니엘관301호(中)강의실</t>
+        </is>
+      </c>
       <c r="L984" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -59083,9 +59399,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I985" t="inlineStr"/>
-      <c r="J985" t="inlineStr"/>
-      <c r="K985" t="inlineStr"/>
+      <c r="I985" t="inlineStr">
+        <is>
+          <t>이정우</t>
+        </is>
+      </c>
+      <c r="J985" t="inlineStr">
+        <is>
+          <t>수6~8</t>
+        </is>
+      </c>
+      <c r="K985" t="inlineStr">
+        <is>
+          <t>바울관203호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L985" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -59139,9 +59467,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I986" t="inlineStr"/>
-      <c r="J986" t="inlineStr"/>
-      <c r="K986" t="inlineStr"/>
+      <c r="I986" t="inlineStr">
+        <is>
+          <t>이동학</t>
+        </is>
+      </c>
+      <c r="J986" t="inlineStr">
+        <is>
+          <t>수5~7</t>
+        </is>
+      </c>
+      <c r="K986" t="inlineStr">
+        <is>
+          <t>요한관221호(中)(교필토익전용)강의실</t>
+        </is>
+      </c>
       <c r="L986" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -59195,9 +59535,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I987" t="inlineStr"/>
-      <c r="J987" t="inlineStr"/>
-      <c r="K987" t="inlineStr"/>
+      <c r="I987" t="inlineStr">
+        <is>
+          <t>강병용</t>
+        </is>
+      </c>
+      <c r="J987" t="inlineStr">
+        <is>
+          <t>수7~9</t>
+        </is>
+      </c>
+      <c r="K987" t="inlineStr">
+        <is>
+          <t>다니엘관306호(中)강의실(첨단강의실)</t>
+        </is>
+      </c>
       <c r="L987" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -59251,9 +59603,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I988" t="inlineStr"/>
-      <c r="J988" t="inlineStr"/>
-      <c r="K988" t="inlineStr"/>
+      <c r="I988" t="inlineStr">
+        <is>
+          <t>권기욱</t>
+        </is>
+      </c>
+      <c r="J988" t="inlineStr">
+        <is>
+          <t>월2~4</t>
+        </is>
+      </c>
+      <c r="K988" t="inlineStr">
+        <is>
+          <t>요한관425호(小)(한국어과정)</t>
+        </is>
+      </c>
       <c r="L988" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -59307,9 +59671,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I989" t="inlineStr"/>
-      <c r="J989" t="inlineStr"/>
-      <c r="K989" t="inlineStr"/>
+      <c r="I989" t="inlineStr">
+        <is>
+          <t>고원배</t>
+        </is>
+      </c>
+      <c r="J989" t="inlineStr">
+        <is>
+          <t>화5~7</t>
+        </is>
+      </c>
+      <c r="K989" t="inlineStr">
+        <is>
+          <t>요한관425호(小)(한국어과정)</t>
+        </is>
+      </c>
       <c r="L989" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -59363,9 +59739,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I990" t="inlineStr"/>
-      <c r="J990" t="inlineStr"/>
-      <c r="K990" t="inlineStr"/>
+      <c r="I990" t="inlineStr">
+        <is>
+          <t>권기욱</t>
+        </is>
+      </c>
+      <c r="J990" t="inlineStr">
+        <is>
+          <t>화6~8</t>
+        </is>
+      </c>
+      <c r="K990" t="inlineStr">
+        <is>
+          <t>요한관223호(中)(교필토익전용)강의실</t>
+        </is>
+      </c>
       <c r="L990" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -59419,9 +59807,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I991" t="inlineStr"/>
-      <c r="J991" t="inlineStr"/>
-      <c r="K991" t="inlineStr"/>
+      <c r="I991" t="inlineStr">
+        <is>
+          <t>Zheng Chengzhe</t>
+        </is>
+      </c>
+      <c r="J991" t="inlineStr">
+        <is>
+          <t>목6~8</t>
+        </is>
+      </c>
+      <c r="K991" t="inlineStr">
+        <is>
+          <t>신학관201호강의실</t>
+        </is>
+      </c>
       <c r="L991" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -59475,9 +59875,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I992" t="inlineStr"/>
-      <c r="J992" t="inlineStr"/>
-      <c r="K992" t="inlineStr"/>
+      <c r="I992" t="inlineStr">
+        <is>
+          <t>김명희</t>
+        </is>
+      </c>
+      <c r="J992" t="inlineStr">
+        <is>
+          <t>수6~8</t>
+        </is>
+      </c>
+      <c r="K992" t="inlineStr">
+        <is>
+          <t>다니엘관402호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L992" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -59531,9 +59943,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I993" t="inlineStr"/>
-      <c r="J993" t="inlineStr"/>
-      <c r="K993" t="inlineStr"/>
+      <c r="I993" t="inlineStr">
+        <is>
+          <t>김비</t>
+        </is>
+      </c>
+      <c r="J993" t="inlineStr">
+        <is>
+          <t>화7~9</t>
+        </is>
+      </c>
+      <c r="K993" t="inlineStr">
+        <is>
+          <t>신학관103호강의실</t>
+        </is>
+      </c>
       <c r="L993" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -59587,9 +60011,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I994" t="inlineStr"/>
-      <c r="J994" t="inlineStr"/>
-      <c r="K994" t="inlineStr"/>
+      <c r="I994" t="inlineStr">
+        <is>
+          <t>김정헌</t>
+        </is>
+      </c>
+      <c r="J994" t="inlineStr">
+        <is>
+          <t>화2~4</t>
+        </is>
+      </c>
+      <c r="K994" t="inlineStr">
+        <is>
+          <t>다니엘관401호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L994" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -59643,7 +60079,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I995" t="inlineStr"/>
+      <c r="I995" t="inlineStr">
+        <is>
+          <t>김선미</t>
+        </is>
+      </c>
       <c r="J995" t="inlineStr"/>
       <c r="K995" t="inlineStr"/>
       <c r="L995" t="inlineStr">
@@ -59699,9 +60139,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I996" t="inlineStr"/>
-      <c r="J996" t="inlineStr"/>
-      <c r="K996" t="inlineStr"/>
+      <c r="I996" t="inlineStr">
+        <is>
+          <t>김선미</t>
+        </is>
+      </c>
+      <c r="J996" t="inlineStr">
+        <is>
+          <t>수4~6</t>
+        </is>
+      </c>
+      <c r="K996" t="inlineStr">
+        <is>
+          <t>사무엘관208호강의실</t>
+        </is>
+      </c>
       <c r="L996" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -59755,7 +60207,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I997" t="inlineStr"/>
+      <c r="I997" t="inlineStr">
+        <is>
+          <t>김선미</t>
+        </is>
+      </c>
       <c r="J997" t="inlineStr"/>
       <c r="K997" t="inlineStr"/>
       <c r="L997" t="inlineStr">
@@ -59811,9 +60267,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I998" t="inlineStr"/>
-      <c r="J998" t="inlineStr"/>
-      <c r="K998" t="inlineStr"/>
+      <c r="I998" t="inlineStr">
+        <is>
+          <t>윤미</t>
+        </is>
+      </c>
+      <c r="J998" t="inlineStr">
+        <is>
+          <t>화4~6</t>
+        </is>
+      </c>
+      <c r="K998" t="inlineStr">
+        <is>
+          <t>사무엘관209호강의실</t>
+        </is>
+      </c>
       <c r="L998" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -59867,9 +60335,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I999" t="inlineStr"/>
-      <c r="J999" t="inlineStr"/>
-      <c r="K999" t="inlineStr"/>
+      <c r="I999" t="inlineStr">
+        <is>
+          <t>허은혜</t>
+        </is>
+      </c>
+      <c r="J999" t="inlineStr">
+        <is>
+          <t>화4~6</t>
+        </is>
+      </c>
+      <c r="K999" t="inlineStr">
+        <is>
+          <t>다니엘관406호(PBL 전용 Lab. 中)강의실</t>
+        </is>
+      </c>
       <c r="L999" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -59923,9 +60403,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1000" t="inlineStr"/>
-      <c r="J1000" t="inlineStr"/>
-      <c r="K1000" t="inlineStr"/>
+      <c r="I1000" t="inlineStr">
+        <is>
+          <t>김미영</t>
+        </is>
+      </c>
+      <c r="J1000" t="inlineStr">
+        <is>
+          <t>목2~4</t>
+        </is>
+      </c>
+      <c r="K1000" t="inlineStr">
+        <is>
+          <t>사무엘관202호강의실</t>
+        </is>
+      </c>
       <c r="L1000" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -59979,9 +60471,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1001" t="inlineStr"/>
-      <c r="J1001" t="inlineStr"/>
-      <c r="K1001" t="inlineStr"/>
+      <c r="I1001" t="inlineStr">
+        <is>
+          <t>김영화</t>
+        </is>
+      </c>
+      <c r="J1001" t="inlineStr">
+        <is>
+          <t>월5~7</t>
+        </is>
+      </c>
+      <c r="K1001" t="inlineStr">
+        <is>
+          <t>요한관425호(小)(한국어과정)</t>
+        </is>
+      </c>
       <c r="L1001" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -60035,9 +60539,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1002" t="inlineStr"/>
-      <c r="J1002" t="inlineStr"/>
-      <c r="K1002" t="inlineStr"/>
+      <c r="I1002" t="inlineStr">
+        <is>
+          <t>음영철</t>
+        </is>
+      </c>
+      <c r="J1002" t="inlineStr">
+        <is>
+          <t>목5~7</t>
+        </is>
+      </c>
+      <c r="K1002" t="inlineStr">
+        <is>
+          <t>바울관403호강의실</t>
+        </is>
+      </c>
       <c r="L1002" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -60091,9 +60607,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1003" t="inlineStr"/>
-      <c r="J1003" t="inlineStr"/>
-      <c r="K1003" t="inlineStr"/>
+      <c r="I1003" t="inlineStr">
+        <is>
+          <t>박은수</t>
+        </is>
+      </c>
+      <c r="J1003" t="inlineStr">
+        <is>
+          <t>월2~4</t>
+        </is>
+      </c>
+      <c r="K1003" t="inlineStr">
+        <is>
+          <t>에스라관314호(컴퓨터실습실)</t>
+        </is>
+      </c>
       <c r="L1003" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -60148,8 +60676,16 @@
         </is>
       </c>
       <c r="I1004" t="inlineStr"/>
-      <c r="J1004" t="inlineStr"/>
-      <c r="K1004" t="inlineStr"/>
+      <c r="J1004" t="inlineStr">
+        <is>
+          <t>월7~9</t>
+        </is>
+      </c>
+      <c r="K1004" t="inlineStr">
+        <is>
+          <t>바울관203호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1004" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -60203,9 +60739,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1005" t="inlineStr"/>
-      <c r="J1005" t="inlineStr"/>
-      <c r="K1005" t="inlineStr"/>
+      <c r="I1005" t="inlineStr">
+        <is>
+          <t>김선이</t>
+        </is>
+      </c>
+      <c r="J1005" t="inlineStr">
+        <is>
+          <t>월3~5</t>
+        </is>
+      </c>
+      <c r="K1005" t="inlineStr">
+        <is>
+          <t>신학관103호강의실</t>
+        </is>
+      </c>
       <c r="L1005" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -60259,9 +60807,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1006" t="inlineStr"/>
-      <c r="J1006" t="inlineStr"/>
-      <c r="K1006" t="inlineStr"/>
+      <c r="I1006" t="inlineStr">
+        <is>
+          <t>음영철</t>
+        </is>
+      </c>
+      <c r="J1006" t="inlineStr">
+        <is>
+          <t>목2~4</t>
+        </is>
+      </c>
+      <c r="K1006" t="inlineStr">
+        <is>
+          <t>다니엘관306호(中)강의실(첨단강의실)</t>
+        </is>
+      </c>
       <c r="L1006" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -60315,9 +60875,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1007" t="inlineStr"/>
-      <c r="J1007" t="inlineStr"/>
-      <c r="K1007" t="inlineStr"/>
+      <c r="I1007" t="inlineStr">
+        <is>
+          <t>김용성</t>
+        </is>
+      </c>
+      <c r="J1007" t="inlineStr">
+        <is>
+          <t>월5~7</t>
+        </is>
+      </c>
+      <c r="K1007" t="inlineStr">
+        <is>
+          <t>사무엘관209호강의실</t>
+        </is>
+      </c>
       <c r="L1007" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -60371,9 +60943,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1008" t="inlineStr"/>
-      <c r="J1008" t="inlineStr"/>
-      <c r="K1008" t="inlineStr"/>
+      <c r="I1008" t="inlineStr">
+        <is>
+          <t>최원재</t>
+        </is>
+      </c>
+      <c r="J1008" t="inlineStr">
+        <is>
+          <t>월2~4</t>
+        </is>
+      </c>
+      <c r="K1008" t="inlineStr">
+        <is>
+          <t>다니엘관302호(中)강의실</t>
+        </is>
+      </c>
       <c r="L1008" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -60427,7 +61011,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1009" t="inlineStr"/>
+      <c r="I1009" t="inlineStr">
+        <is>
+          <t>백숭기</t>
+        </is>
+      </c>
       <c r="J1009" t="inlineStr"/>
       <c r="K1009" t="inlineStr"/>
       <c r="L1009" t="inlineStr">
@@ -60483,9 +61071,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1010" t="inlineStr"/>
-      <c r="J1010" t="inlineStr"/>
-      <c r="K1010" t="inlineStr"/>
+      <c r="I1010" t="inlineStr">
+        <is>
+          <t>김정헌</t>
+        </is>
+      </c>
+      <c r="J1010" t="inlineStr">
+        <is>
+          <t>목2~4</t>
+        </is>
+      </c>
+      <c r="K1010" t="inlineStr">
+        <is>
+          <t>다니엘관403호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1010" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -60539,9 +61139,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1011" t="inlineStr"/>
-      <c r="J1011" t="inlineStr"/>
-      <c r="K1011" t="inlineStr"/>
+      <c r="I1011" t="inlineStr">
+        <is>
+          <t>하임성</t>
+        </is>
+      </c>
+      <c r="J1011" t="inlineStr">
+        <is>
+          <t>월7~9</t>
+        </is>
+      </c>
+      <c r="K1011" t="inlineStr">
+        <is>
+          <t>사무엘관201호강의실</t>
+        </is>
+      </c>
       <c r="L1011" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -60595,9 +61207,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1012" t="inlineStr"/>
-      <c r="J1012" t="inlineStr"/>
-      <c r="K1012" t="inlineStr"/>
+      <c r="I1012" t="inlineStr">
+        <is>
+          <t>이양진</t>
+        </is>
+      </c>
+      <c r="J1012" t="inlineStr">
+        <is>
+          <t>수1~3</t>
+        </is>
+      </c>
+      <c r="K1012" t="inlineStr">
+        <is>
+          <t>에스라관406호강의실(첨단강의실)</t>
+        </is>
+      </c>
       <c r="L1012" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -60651,9 +61275,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1013" t="inlineStr"/>
-      <c r="J1013" t="inlineStr"/>
-      <c r="K1013" t="inlineStr"/>
+      <c r="I1013" t="inlineStr">
+        <is>
+          <t>Lee Jeeny Jeeyoun</t>
+        </is>
+      </c>
+      <c r="J1013" t="inlineStr">
+        <is>
+          <t>월6~8</t>
+        </is>
+      </c>
+      <c r="K1013" t="inlineStr">
+        <is>
+          <t>에스라관406호강의실(첨단강의실)</t>
+        </is>
+      </c>
       <c r="L1013" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -60707,9 +61343,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1014" t="inlineStr"/>
-      <c r="J1014" t="inlineStr"/>
-      <c r="K1014" t="inlineStr"/>
+      <c r="I1014" t="inlineStr">
+        <is>
+          <t>이관호</t>
+        </is>
+      </c>
+      <c r="J1014" t="inlineStr">
+        <is>
+          <t>월6~8</t>
+        </is>
+      </c>
+      <c r="K1014" t="inlineStr">
+        <is>
+          <t>다니엘관401호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1014" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -60831,9 +61479,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1016" t="inlineStr"/>
-      <c r="J1016" t="inlineStr"/>
-      <c r="K1016" t="inlineStr"/>
+      <c r="I1016" t="inlineStr">
+        <is>
+          <t>한금윤</t>
+        </is>
+      </c>
+      <c r="J1016" t="inlineStr">
+        <is>
+          <t>화5~7</t>
+        </is>
+      </c>
+      <c r="K1016" t="inlineStr">
+        <is>
+          <t>바울관202호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1016" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -60887,9 +61547,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1017" t="inlineStr"/>
-      <c r="J1017" t="inlineStr"/>
-      <c r="K1017" t="inlineStr"/>
+      <c r="I1017" t="inlineStr">
+        <is>
+          <t>한금윤</t>
+        </is>
+      </c>
+      <c r="J1017" t="inlineStr">
+        <is>
+          <t>월5~7</t>
+        </is>
+      </c>
+      <c r="K1017" t="inlineStr">
+        <is>
+          <t>사무엘관110호강의실</t>
+        </is>
+      </c>
       <c r="L1017" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -60943,9 +61615,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1018" t="inlineStr"/>
-      <c r="J1018" t="inlineStr"/>
-      <c r="K1018" t="inlineStr"/>
+      <c r="I1018" t="inlineStr">
+        <is>
+          <t>최가형</t>
+        </is>
+      </c>
+      <c r="J1018" t="inlineStr">
+        <is>
+          <t>목2~4</t>
+        </is>
+      </c>
+      <c r="K1018" t="inlineStr">
+        <is>
+          <t>사무엘관208호강의실</t>
+        </is>
+      </c>
       <c r="L1018" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -60999,9 +61683,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1019" t="inlineStr"/>
-      <c r="J1019" t="inlineStr"/>
-      <c r="K1019" t="inlineStr"/>
+      <c r="I1019" t="inlineStr">
+        <is>
+          <t>최가형</t>
+        </is>
+      </c>
+      <c r="J1019" t="inlineStr">
+        <is>
+          <t>수2~4</t>
+        </is>
+      </c>
+      <c r="K1019" t="inlineStr">
+        <is>
+          <t>사무엘관108호(PBL소형)강의실</t>
+        </is>
+      </c>
       <c r="L1019" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -61055,9 +61751,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1020" t="inlineStr"/>
-      <c r="J1020" t="inlineStr"/>
-      <c r="K1020" t="inlineStr"/>
+      <c r="I1020" t="inlineStr">
+        <is>
+          <t>전지은</t>
+        </is>
+      </c>
+      <c r="J1020" t="inlineStr">
+        <is>
+          <t>목4~6</t>
+        </is>
+      </c>
+      <c r="K1020" t="inlineStr">
+        <is>
+          <t>사무엘관210호(PBL소형)강의실</t>
+        </is>
+      </c>
       <c r="L1020" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -61111,9 +61819,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1021" t="inlineStr"/>
-      <c r="J1021" t="inlineStr"/>
-      <c r="K1021" t="inlineStr"/>
+      <c r="I1021" t="inlineStr">
+        <is>
+          <t>전지은</t>
+        </is>
+      </c>
+      <c r="J1021" t="inlineStr">
+        <is>
+          <t>목1~3</t>
+        </is>
+      </c>
+      <c r="K1021" t="inlineStr">
+        <is>
+          <t>사무엘관210호(PBL소형)강의실</t>
+        </is>
+      </c>
       <c r="L1021" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -61167,9 +61887,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1022" t="inlineStr"/>
-      <c r="J1022" t="inlineStr"/>
-      <c r="K1022" t="inlineStr"/>
+      <c r="I1022" t="inlineStr">
+        <is>
+          <t>임준서</t>
+        </is>
+      </c>
+      <c r="J1022" t="inlineStr">
+        <is>
+          <t>목6~8</t>
+        </is>
+      </c>
+      <c r="K1022" t="inlineStr">
+        <is>
+          <t>바울관202호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1022" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -61223,9 +61955,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1023" t="inlineStr"/>
-      <c r="J1023" t="inlineStr"/>
-      <c r="K1023" t="inlineStr"/>
+      <c r="I1023" t="inlineStr">
+        <is>
+          <t>임준서</t>
+        </is>
+      </c>
+      <c r="J1023" t="inlineStr">
+        <is>
+          <t>목2~4</t>
+        </is>
+      </c>
+      <c r="K1023" t="inlineStr">
+        <is>
+          <t>바울관202호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1023" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -61279,9 +62023,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1024" t="inlineStr"/>
-      <c r="J1024" t="inlineStr"/>
-      <c r="K1024" t="inlineStr"/>
+      <c r="I1024" t="inlineStr">
+        <is>
+          <t>이관호</t>
+        </is>
+      </c>
+      <c r="J1024" t="inlineStr">
+        <is>
+          <t>월3~5</t>
+        </is>
+      </c>
+      <c r="K1024" t="inlineStr">
+        <is>
+          <t>다니엘관401호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1024" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -61335,8 +62091,16 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1025" t="inlineStr"/>
-      <c r="J1025" t="inlineStr"/>
+      <c r="I1025" t="inlineStr">
+        <is>
+          <t>유승현</t>
+        </is>
+      </c>
+      <c r="J1025" t="inlineStr">
+        <is>
+          <t>수5~7</t>
+        </is>
+      </c>
       <c r="K1025" t="inlineStr"/>
       <c r="L1025" t="inlineStr">
         <is>
@@ -61391,8 +62155,16 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1026" t="inlineStr"/>
-      <c r="J1026" t="inlineStr"/>
+      <c r="I1026" t="inlineStr">
+        <is>
+          <t>유승현</t>
+        </is>
+      </c>
+      <c r="J1026" t="inlineStr">
+        <is>
+          <t>수2~4</t>
+        </is>
+      </c>
       <c r="K1026" t="inlineStr"/>
       <c r="L1026" t="inlineStr">
         <is>
@@ -61447,9 +62219,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1027" t="inlineStr"/>
-      <c r="J1027" t="inlineStr"/>
-      <c r="K1027" t="inlineStr"/>
+      <c r="I1027" t="inlineStr">
+        <is>
+          <t>박성준</t>
+        </is>
+      </c>
+      <c r="J1027" t="inlineStr">
+        <is>
+          <t>수5~7</t>
+        </is>
+      </c>
+      <c r="K1027" t="inlineStr">
+        <is>
+          <t>요한관425호(小)(한국어과정)</t>
+        </is>
+      </c>
       <c r="L1027" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -61503,9 +62287,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1028" t="inlineStr"/>
-      <c r="J1028" t="inlineStr"/>
-      <c r="K1028" t="inlineStr"/>
+      <c r="I1028" t="inlineStr">
+        <is>
+          <t>박성준</t>
+        </is>
+      </c>
+      <c r="J1028" t="inlineStr">
+        <is>
+          <t>수2~4</t>
+        </is>
+      </c>
+      <c r="K1028" t="inlineStr">
+        <is>
+          <t>다니엘관406호(PBL 전용 Lab. 中)강의실</t>
+        </is>
+      </c>
       <c r="L1028" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -61559,9 +62355,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1029" t="inlineStr"/>
-      <c r="J1029" t="inlineStr"/>
-      <c r="K1029" t="inlineStr"/>
+      <c r="I1029" t="inlineStr">
+        <is>
+          <t>김정헌</t>
+        </is>
+      </c>
+      <c r="J1029" t="inlineStr">
+        <is>
+          <t>월6~8</t>
+        </is>
+      </c>
+      <c r="K1029" t="inlineStr">
+        <is>
+          <t>다니엘관406호(PBL 전용 Lab. 中)강의실</t>
+        </is>
+      </c>
       <c r="L1029" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -61615,9 +62423,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1030" t="inlineStr"/>
-      <c r="J1030" t="inlineStr"/>
-      <c r="K1030" t="inlineStr"/>
+      <c r="I1030" t="inlineStr">
+        <is>
+          <t>김정헌</t>
+        </is>
+      </c>
+      <c r="J1030" t="inlineStr">
+        <is>
+          <t>월2~4</t>
+        </is>
+      </c>
+      <c r="K1030" t="inlineStr">
+        <is>
+          <t>다니엘관406호(PBL 전용 Lab. 中)강의실</t>
+        </is>
+      </c>
       <c r="L1030" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -61671,9 +62491,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1031" t="inlineStr"/>
-      <c r="J1031" t="inlineStr"/>
-      <c r="K1031" t="inlineStr"/>
+      <c r="I1031" t="inlineStr">
+        <is>
+          <t>권도경</t>
+        </is>
+      </c>
+      <c r="J1031" t="inlineStr">
+        <is>
+          <t>수4~6</t>
+        </is>
+      </c>
+      <c r="K1031" t="inlineStr">
+        <is>
+          <t>바울관202호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1031" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -61727,9 +62559,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1032" t="inlineStr"/>
-      <c r="J1032" t="inlineStr"/>
-      <c r="K1032" t="inlineStr"/>
+      <c r="I1032" t="inlineStr">
+        <is>
+          <t>권도경</t>
+        </is>
+      </c>
+      <c r="J1032" t="inlineStr">
+        <is>
+          <t>수1~3</t>
+        </is>
+      </c>
+      <c r="K1032" t="inlineStr">
+        <is>
+          <t>사무엘관109호강의실</t>
+        </is>
+      </c>
       <c r="L1032" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -61783,9 +62627,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1033" t="inlineStr"/>
-      <c r="J1033" t="inlineStr"/>
-      <c r="K1033" t="inlineStr"/>
+      <c r="I1033" t="inlineStr">
+        <is>
+          <t>한금윤</t>
+        </is>
+      </c>
+      <c r="J1033" t="inlineStr">
+        <is>
+          <t>수2~4</t>
+        </is>
+      </c>
+      <c r="K1033" t="inlineStr">
+        <is>
+          <t>사무엘관201호강의실</t>
+        </is>
+      </c>
       <c r="L1033" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -61839,9 +62695,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1034" t="inlineStr"/>
-      <c r="J1034" t="inlineStr"/>
-      <c r="K1034" t="inlineStr"/>
+      <c r="I1034" t="inlineStr">
+        <is>
+          <t>김훈</t>
+        </is>
+      </c>
+      <c r="J1034" t="inlineStr">
+        <is>
+          <t>수7~9</t>
+        </is>
+      </c>
+      <c r="K1034" t="inlineStr">
+        <is>
+          <t>요한관222호(中)(교필토익전용)강의실</t>
+        </is>
+      </c>
       <c r="L1034" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -61895,9 +62763,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1035" t="inlineStr"/>
-      <c r="J1035" t="inlineStr"/>
-      <c r="K1035" t="inlineStr"/>
+      <c r="I1035" t="inlineStr">
+        <is>
+          <t>김훈</t>
+        </is>
+      </c>
+      <c r="J1035" t="inlineStr">
+        <is>
+          <t>목7~9</t>
+        </is>
+      </c>
+      <c r="K1035" t="inlineStr">
+        <is>
+          <t>요한관224호(中)강의실</t>
+        </is>
+      </c>
       <c r="L1035" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -61951,9 +62831,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1036" t="inlineStr"/>
-      <c r="J1036" t="inlineStr"/>
-      <c r="K1036" t="inlineStr"/>
+      <c r="I1036" t="inlineStr">
+        <is>
+          <t>류기현</t>
+        </is>
+      </c>
+      <c r="J1036" t="inlineStr">
+        <is>
+          <t>화5~7</t>
+        </is>
+      </c>
+      <c r="K1036" t="inlineStr">
+        <is>
+          <t>신학관210호강의실</t>
+        </is>
+      </c>
       <c r="L1036" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -62007,9 +62899,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1037" t="inlineStr"/>
-      <c r="J1037" t="inlineStr"/>
-      <c r="K1037" t="inlineStr"/>
+      <c r="I1037" t="inlineStr">
+        <is>
+          <t>명지원</t>
+        </is>
+      </c>
+      <c r="J1037" t="inlineStr">
+        <is>
+          <t>목5~7</t>
+        </is>
+      </c>
+      <c r="K1037" t="inlineStr">
+        <is>
+          <t>요한관221호(中)(교필토익전용)강의실</t>
+        </is>
+      </c>
       <c r="L1037" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -62063,8 +62967,16 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1038" t="inlineStr"/>
-      <c r="J1038" t="inlineStr"/>
+      <c r="I1038" t="inlineStr">
+        <is>
+          <t>김의석</t>
+        </is>
+      </c>
+      <c r="J1038" t="inlineStr">
+        <is>
+          <t>월7~9</t>
+        </is>
+      </c>
       <c r="K1038" t="inlineStr"/>
       <c r="L1038" t="inlineStr">
         <is>
@@ -62119,9 +63031,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1039" t="inlineStr"/>
-      <c r="J1039" t="inlineStr"/>
-      <c r="K1039" t="inlineStr"/>
+      <c r="I1039" t="inlineStr">
+        <is>
+          <t>고정원</t>
+        </is>
+      </c>
+      <c r="J1039" t="inlineStr">
+        <is>
+          <t>수6~8</t>
+        </is>
+      </c>
+      <c r="K1039" t="inlineStr">
+        <is>
+          <t>사무엘관202호강의실</t>
+        </is>
+      </c>
       <c r="L1039" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -62175,9 +63099,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1040" t="inlineStr"/>
-      <c r="J1040" t="inlineStr"/>
-      <c r="K1040" t="inlineStr"/>
+      <c r="I1040" t="inlineStr">
+        <is>
+          <t>취업정보</t>
+        </is>
+      </c>
+      <c r="J1040" t="inlineStr">
+        <is>
+          <t>수2~4</t>
+        </is>
+      </c>
+      <c r="K1040" t="inlineStr">
+        <is>
+          <t>바울관203호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1040" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -62231,9 +63167,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1041" t="inlineStr"/>
-      <c r="J1041" t="inlineStr"/>
-      <c r="K1041" t="inlineStr"/>
+      <c r="I1041" t="inlineStr">
+        <is>
+          <t>김민주</t>
+        </is>
+      </c>
+      <c r="J1041" t="inlineStr">
+        <is>
+          <t>화2~4</t>
+        </is>
+      </c>
+      <c r="K1041" t="inlineStr">
+        <is>
+          <t>다니엘관402호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1041" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -62287,9 +63235,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1042" t="inlineStr"/>
-      <c r="J1042" t="inlineStr"/>
-      <c r="K1042" t="inlineStr"/>
+      <c r="I1042" t="inlineStr">
+        <is>
+          <t>노동욱</t>
+        </is>
+      </c>
+      <c r="J1042" t="inlineStr">
+        <is>
+          <t>월6~8</t>
+        </is>
+      </c>
+      <c r="K1042" t="inlineStr">
+        <is>
+          <t>요한관222호(中)(교필토익전용)강의실</t>
+        </is>
+      </c>
       <c r="L1042" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -62343,9 +63303,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1043" t="inlineStr"/>
-      <c r="J1043" t="inlineStr"/>
-      <c r="K1043" t="inlineStr"/>
+      <c r="I1043" t="inlineStr">
+        <is>
+          <t>최수동</t>
+        </is>
+      </c>
+      <c r="J1043" t="inlineStr">
+        <is>
+          <t>화6~8</t>
+        </is>
+      </c>
+      <c r="K1043" t="inlineStr">
+        <is>
+          <t>요한관221호(中)(교필토익전용)강의실</t>
+        </is>
+      </c>
       <c r="L1043" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -62399,9 +63371,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1044" t="inlineStr"/>
-      <c r="J1044" t="inlineStr"/>
-      <c r="K1044" t="inlineStr"/>
+      <c r="I1044" t="inlineStr">
+        <is>
+          <t>곽주화</t>
+        </is>
+      </c>
+      <c r="J1044" t="inlineStr">
+        <is>
+          <t>화11~13</t>
+        </is>
+      </c>
+      <c r="K1044" t="inlineStr">
+        <is>
+          <t>신학관202호강의실(PBL)</t>
+        </is>
+      </c>
       <c r="L1044" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -62455,9 +63439,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1045" t="inlineStr"/>
-      <c r="J1045" t="inlineStr"/>
-      <c r="K1045" t="inlineStr"/>
+      <c r="I1045" t="inlineStr">
+        <is>
+          <t>신동진</t>
+        </is>
+      </c>
+      <c r="J1045" t="inlineStr">
+        <is>
+          <t>월5~7</t>
+        </is>
+      </c>
+      <c r="K1045" t="inlineStr">
+        <is>
+          <t>에스라관210호강의실</t>
+        </is>
+      </c>
       <c r="L1045" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -62511,9 +63507,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1046" t="inlineStr"/>
-      <c r="J1046" t="inlineStr"/>
-      <c r="K1046" t="inlineStr"/>
+      <c r="I1046" t="inlineStr">
+        <is>
+          <t>강동균</t>
+        </is>
+      </c>
+      <c r="J1046" t="inlineStr">
+        <is>
+          <t>목6~8</t>
+        </is>
+      </c>
+      <c r="K1046" t="inlineStr">
+        <is>
+          <t>사무엘관110호강의실</t>
+        </is>
+      </c>
       <c r="L1046" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -62635,9 +63643,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1048" t="inlineStr"/>
-      <c r="J1048" t="inlineStr"/>
-      <c r="K1048" t="inlineStr"/>
+      <c r="I1048" t="inlineStr">
+        <is>
+          <t>박승순</t>
+        </is>
+      </c>
+      <c r="J1048" t="inlineStr">
+        <is>
+          <t>화4~6</t>
+        </is>
+      </c>
+      <c r="K1048" t="inlineStr">
+        <is>
+          <t>체육관 108(세미나실)</t>
+        </is>
+      </c>
       <c r="L1048" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -62691,9 +63711,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1049" t="inlineStr"/>
-      <c r="J1049" t="inlineStr"/>
-      <c r="K1049" t="inlineStr"/>
+      <c r="I1049" t="inlineStr">
+        <is>
+          <t>윤미</t>
+        </is>
+      </c>
+      <c r="J1049" t="inlineStr">
+        <is>
+          <t>화1~3</t>
+        </is>
+      </c>
+      <c r="K1049" t="inlineStr">
+        <is>
+          <t>사무엘관109호강의실</t>
+        </is>
+      </c>
       <c r="L1049" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -62747,9 +63779,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1050" t="inlineStr"/>
-      <c r="J1050" t="inlineStr"/>
-      <c r="K1050" t="inlineStr"/>
+      <c r="I1050" t="inlineStr">
+        <is>
+          <t>윤미</t>
+        </is>
+      </c>
+      <c r="J1050" t="inlineStr">
+        <is>
+          <t>월2~4</t>
+        </is>
+      </c>
+      <c r="K1050" t="inlineStr">
+        <is>
+          <t>에스라관209호강의실(교직과목)(첨단강의실)</t>
+        </is>
+      </c>
       <c r="L1050" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -62803,9 +63847,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1051" t="inlineStr"/>
-      <c r="J1051" t="inlineStr"/>
-      <c r="K1051" t="inlineStr"/>
+      <c r="I1051" t="inlineStr">
+        <is>
+          <t>정재신</t>
+        </is>
+      </c>
+      <c r="J1051" t="inlineStr">
+        <is>
+          <t>월7~9</t>
+        </is>
+      </c>
+      <c r="K1051" t="inlineStr">
+        <is>
+          <t>신학관103호강의실</t>
+        </is>
+      </c>
       <c r="L1051" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -62859,9 +63915,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1052" t="inlineStr"/>
-      <c r="J1052" t="inlineStr"/>
-      <c r="K1052" t="inlineStr"/>
+      <c r="I1052" t="inlineStr">
+        <is>
+          <t>김정헌</t>
+        </is>
+      </c>
+      <c r="J1052" t="inlineStr">
+        <is>
+          <t>수2~4</t>
+        </is>
+      </c>
+      <c r="K1052" t="inlineStr">
+        <is>
+          <t>다니엘관402호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1052" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -62915,9 +63983,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1053" t="inlineStr"/>
-      <c r="J1053" t="inlineStr"/>
-      <c r="K1053" t="inlineStr"/>
+      <c r="I1053" t="inlineStr">
+        <is>
+          <t>김용성</t>
+        </is>
+      </c>
+      <c r="J1053" t="inlineStr">
+        <is>
+          <t>화5~7</t>
+        </is>
+      </c>
+      <c r="K1053" t="inlineStr">
+        <is>
+          <t>요한관222호(中)(교필토익전용)강의실</t>
+        </is>
+      </c>
       <c r="L1053" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -62971,9 +64051,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1054" t="inlineStr"/>
-      <c r="J1054" t="inlineStr"/>
-      <c r="K1054" t="inlineStr"/>
+      <c r="I1054" t="inlineStr">
+        <is>
+          <t>홍선미</t>
+        </is>
+      </c>
+      <c r="J1054" t="inlineStr">
+        <is>
+          <t>수5~7</t>
+        </is>
+      </c>
+      <c r="K1054" t="inlineStr">
+        <is>
+          <t>신학관210호강의실</t>
+        </is>
+      </c>
       <c r="L1054" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -63027,7 +64119,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1055" t="inlineStr"/>
+      <c r="I1055" t="inlineStr">
+        <is>
+          <t>로즈마리신</t>
+        </is>
+      </c>
       <c r="J1055" t="inlineStr"/>
       <c r="K1055" t="inlineStr"/>
       <c r="L1055" t="inlineStr">
@@ -63083,9 +64179,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1056" t="inlineStr"/>
-      <c r="J1056" t="inlineStr"/>
-      <c r="K1056" t="inlineStr"/>
+      <c r="I1056" t="inlineStr">
+        <is>
+          <t>Alexander Park</t>
+        </is>
+      </c>
+      <c r="J1056" t="inlineStr">
+        <is>
+          <t>목7~9</t>
+        </is>
+      </c>
+      <c r="K1056" t="inlineStr">
+        <is>
+          <t>사무엘관201호강의실</t>
+        </is>
+      </c>
       <c r="L1056" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -63139,9 +64247,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1057" t="inlineStr"/>
-      <c r="J1057" t="inlineStr"/>
-      <c r="K1057" t="inlineStr"/>
+      <c r="I1057" t="inlineStr">
+        <is>
+          <t>김형태</t>
+        </is>
+      </c>
+      <c r="J1057" t="inlineStr">
+        <is>
+          <t>화6~8</t>
+        </is>
+      </c>
+      <c r="K1057" t="inlineStr">
+        <is>
+          <t>다니엘관401호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1057" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -63195,9 +64315,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1058" t="inlineStr"/>
-      <c r="J1058" t="inlineStr"/>
-      <c r="K1058" t="inlineStr"/>
+      <c r="I1058" t="inlineStr">
+        <is>
+          <t>한금윤</t>
+        </is>
+      </c>
+      <c r="J1058" t="inlineStr">
+        <is>
+          <t>수5~7</t>
+        </is>
+      </c>
+      <c r="K1058" t="inlineStr">
+        <is>
+          <t>사무엘관110호강의실</t>
+        </is>
+      </c>
       <c r="L1058" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -63251,9 +64383,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1059" t="inlineStr"/>
-      <c r="J1059" t="inlineStr"/>
-      <c r="K1059" t="inlineStr"/>
+      <c r="I1059" t="inlineStr">
+        <is>
+          <t>김나미</t>
+        </is>
+      </c>
+      <c r="J1059" t="inlineStr">
+        <is>
+          <t>수7~9</t>
+        </is>
+      </c>
+      <c r="K1059" t="inlineStr">
+        <is>
+          <t>에스라관406호강의실(첨단강의실)</t>
+        </is>
+      </c>
       <c r="L1059" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -63307,9 +64451,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1060" t="inlineStr"/>
-      <c r="J1060" t="inlineStr"/>
-      <c r="K1060" t="inlineStr"/>
+      <c r="I1060" t="inlineStr">
+        <is>
+          <t>이미희</t>
+        </is>
+      </c>
+      <c r="J1060" t="inlineStr">
+        <is>
+          <t>목2~4</t>
+        </is>
+      </c>
+      <c r="K1060" t="inlineStr">
+        <is>
+          <t>다니엘관401호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1060" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -63363,9 +64519,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1061" t="inlineStr"/>
-      <c r="J1061" t="inlineStr"/>
-      <c r="K1061" t="inlineStr"/>
+      <c r="I1061" t="inlineStr">
+        <is>
+          <t>김현정</t>
+        </is>
+      </c>
+      <c r="J1061" t="inlineStr">
+        <is>
+          <t>수2~4</t>
+        </is>
+      </c>
+      <c r="K1061" t="inlineStr">
+        <is>
+          <t>다니엘관403호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1061" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -63419,9 +64587,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1062" t="inlineStr"/>
-      <c r="J1062" t="inlineStr"/>
-      <c r="K1062" t="inlineStr"/>
+      <c r="I1062" t="inlineStr">
+        <is>
+          <t>김동건</t>
+        </is>
+      </c>
+      <c r="J1062" t="inlineStr">
+        <is>
+          <t>월1~3</t>
+        </is>
+      </c>
+      <c r="K1062" t="inlineStr">
+        <is>
+          <t>다니엘관402호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1062" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -63475,9 +64655,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1063" t="inlineStr"/>
-      <c r="J1063" t="inlineStr"/>
-      <c r="K1063" t="inlineStr"/>
+      <c r="I1063" t="inlineStr">
+        <is>
+          <t>강병용</t>
+        </is>
+      </c>
+      <c r="J1063" t="inlineStr">
+        <is>
+          <t>목7~9</t>
+        </is>
+      </c>
+      <c r="K1063" t="inlineStr">
+        <is>
+          <t>다니엘관403호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1063" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -63531,9 +64723,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1064" t="inlineStr"/>
-      <c r="J1064" t="inlineStr"/>
-      <c r="K1064" t="inlineStr"/>
+      <c r="I1064" t="inlineStr">
+        <is>
+          <t>최원재</t>
+        </is>
+      </c>
+      <c r="J1064" t="inlineStr">
+        <is>
+          <t>월5~7</t>
+        </is>
+      </c>
+      <c r="K1064" t="inlineStr">
+        <is>
+          <t>요한관223호(中)(교필토익전용)강의실</t>
+        </is>
+      </c>
       <c r="L1064" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -63587,9 +64791,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1065" t="inlineStr"/>
-      <c r="J1065" t="inlineStr"/>
-      <c r="K1065" t="inlineStr"/>
+      <c r="I1065" t="inlineStr">
+        <is>
+          <t>안병삼</t>
+        </is>
+      </c>
+      <c r="J1065" t="inlineStr">
+        <is>
+          <t>화5~7</t>
+        </is>
+      </c>
+      <c r="K1065" t="inlineStr">
+        <is>
+          <t>요한관326호(小)강의실(한국어과정)</t>
+        </is>
+      </c>
       <c r="L1065" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -63643,9 +64859,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1066" t="inlineStr"/>
-      <c r="J1066" t="inlineStr"/>
-      <c r="K1066" t="inlineStr"/>
+      <c r="I1066" t="inlineStr">
+        <is>
+          <t>이현재</t>
+        </is>
+      </c>
+      <c r="J1066" t="inlineStr">
+        <is>
+          <t>화5~7</t>
+        </is>
+      </c>
+      <c r="K1066" t="inlineStr">
+        <is>
+          <t>다니엘관403호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1066" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -63699,9 +64927,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1067" t="inlineStr"/>
-      <c r="J1067" t="inlineStr"/>
-      <c r="K1067" t="inlineStr"/>
+      <c r="I1067" t="inlineStr">
+        <is>
+          <t>이현재</t>
+        </is>
+      </c>
+      <c r="J1067" t="inlineStr">
+        <is>
+          <t>월5~7</t>
+        </is>
+      </c>
+      <c r="K1067" t="inlineStr">
+        <is>
+          <t>다니엘관403호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1067" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -63755,9 +64995,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1068" t="inlineStr"/>
-      <c r="J1068" t="inlineStr"/>
-      <c r="K1068" t="inlineStr"/>
+      <c r="I1068" t="inlineStr">
+        <is>
+          <t>김도영</t>
+        </is>
+      </c>
+      <c r="J1068" t="inlineStr">
+        <is>
+          <t>수7~9</t>
+        </is>
+      </c>
+      <c r="K1068" t="inlineStr">
+        <is>
+          <t>요한관421호(中)강의실</t>
+        </is>
+      </c>
       <c r="L1068" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -63811,7 +65063,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1069" t="inlineStr"/>
+      <c r="I1069" t="inlineStr">
+        <is>
+          <t>박민수</t>
+        </is>
+      </c>
       <c r="J1069" t="inlineStr"/>
       <c r="K1069" t="inlineStr"/>
       <c r="L1069" t="inlineStr">
@@ -64271,9 +65527,21 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I1077" t="inlineStr"/>
-      <c r="J1077" t="inlineStr"/>
-      <c r="K1077" t="inlineStr"/>
+      <c r="I1077" t="inlineStr">
+        <is>
+          <t>김현정</t>
+        </is>
+      </c>
+      <c r="J1077" t="inlineStr">
+        <is>
+          <t>수6~8</t>
+        </is>
+      </c>
+      <c r="K1077" t="inlineStr">
+        <is>
+          <t>다니엘관403호(PBL)강의실</t>
+        </is>
+      </c>
       <c r="L1077" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -70399,7 +71667,7 @@
       </c>
       <c r="K1179" t="inlineStr">
         <is>
-          <t>에스라관113호강의실</t>
+          <t>미지정</t>
         </is>
       </c>
       <c r="L1179" t="inlineStr">
@@ -71435,7 +72703,7 @@
       </c>
       <c r="K1196" t="inlineStr">
         <is>
-          <t>에스라관406호강의실(첨단강의실)</t>
+          <t>아트앤디자인202호강의실</t>
         </is>
       </c>
       <c r="L1196" t="inlineStr">
@@ -72895,7 +74163,7 @@
       </c>
       <c r="K1220" t="inlineStr">
         <is>
-          <t>디자인관113호(일러스트스튜디오1)</t>
+          <t>아트앤디자인202호강의실</t>
         </is>
       </c>
       <c r="L1220" t="inlineStr">
@@ -74346,12 +75614,12 @@
       </c>
       <c r="J1244" t="inlineStr">
         <is>
-          <t>월2~3</t>
+          <t>수5~6</t>
         </is>
       </c>
       <c r="K1244" t="inlineStr">
         <is>
-          <t>아트앤디자인206호강의실(미컨실험실습실)</t>
+          <t>아트앤디자인202호강의실</t>
         </is>
       </c>
       <c r="L1244" t="inlineStr">
@@ -84967,7 +86235,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="I1419" t="inlineStr"/>
+      <c r="I1419" t="inlineStr">
+        <is>
+          <t>미지정</t>
+        </is>
+      </c>
       <c r="J1419" t="inlineStr">
         <is>
           <t>월7~8</t>

</xml_diff>

<commit_message>
chore(data): add 2026-2 data files ('26.07.18)
</commit_message>
<xml_diff>
--- a/data/2026년 2학기 정규 시간표.xlsx
+++ b/data/2026년 2학기 정규 시간표.xlsx
@@ -1619,7 +1619,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>미지정</t>
+          <t>다니엘관402호(PBL)강의실</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>미지정</t>
+          <t>다니엘관403호(PBL)강의실</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>미지정</t>
+          <t>다니엘관401호(PBL)강의실</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>제3과학관207호강의실</t>
+          <t>다니엘관306호(中)강의실(첨단강의실)</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>다니엘관208호(大)강의실</t>
+          <t>제3과학관207호강의실</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -3151,7 +3151,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>요한관323호(中)강의실</t>
+          <t>제3과학관207호강의실</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>다니엘관404호(大)강의실,요한관323호(中)강의실</t>
+          <t>다니엘관208호(大)강의실,다니엘관404호(大)강의실</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -3794,12 +3794,12 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>수8~9,목10~11</t>
+          <t>수8~9,목1~2</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>다니엘관404호(大)강의실</t>
+          <t>다니엘관404호(大)강의실,다니엘관405호(大)강의실</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -4375,7 +4375,7 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>다니엘관404호(大)강의실</t>
+          <t>제3과학관207호강의실</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -7431,7 +7431,7 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>미지정</t>
+          <t>다니엘관304호(大)</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
@@ -7835,7 +7835,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>미지정</t>
+          <t>신학관404호(배창현기념관)</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
@@ -11155,7 +11155,7 @@
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>미지정</t>
+          <t>신학관404호(배창현기념관)</t>
         </is>
       </c>
       <c r="L188" t="inlineStr">
@@ -17217,7 +17217,11 @@
           <t>월5~8</t>
         </is>
       </c>
-      <c r="K290" t="inlineStr"/>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>요한관423호(中)강의실</t>
+        </is>
+      </c>
       <c r="L290" t="inlineStr">
         <is>
           <t>미래융합대학</t>
@@ -18295,7 +18299,7 @@
       </c>
       <c r="K308" t="inlineStr">
         <is>
-          <t>다니엘관306호(中)강의실(첨단강의실)</t>
+          <t>다니엘관B101호(大)(자유전공학부 전용)</t>
         </is>
       </c>
       <c r="L308" t="inlineStr">
@@ -20147,7 +20151,7 @@
       </c>
       <c r="K338" t="inlineStr">
         <is>
-          <t>요한관322호(中)강의실</t>
+          <t>국제교육관221호(中)강의실</t>
         </is>
       </c>
       <c r="L338" t="inlineStr">
@@ -20382,12 +20386,12 @@
       </c>
       <c r="J342" t="inlineStr">
         <is>
-          <t>월6~8</t>
+          <t>목6~8</t>
         </is>
       </c>
       <c r="K342" t="inlineStr">
         <is>
-          <t>백주년311호강의실</t>
+          <t>요한관322호(中)강의실</t>
         </is>
       </c>
       <c r="L342" t="inlineStr">
@@ -20442,7 +20446,7 @@
       </c>
       <c r="J343" t="inlineStr">
         <is>
-          <t>목6~8</t>
+          <t>화6~8</t>
         </is>
       </c>
       <c r="K343" t="inlineStr">
@@ -20627,7 +20631,7 @@
       </c>
       <c r="K346" t="inlineStr">
         <is>
-          <t>다니엘관305호(大)</t>
+          <t>바울관214호강의실</t>
         </is>
       </c>
       <c r="L346" t="inlineStr">
@@ -22757,7 +22761,11 @@
           <t>목2~4</t>
         </is>
       </c>
-      <c r="K381" t="inlineStr"/>
+      <c r="K381" t="inlineStr">
+        <is>
+          <t>요한관423호(中)강의실</t>
+        </is>
+      </c>
       <c r="L381" t="inlineStr">
         <is>
           <t>미래융합대학</t>
@@ -33443,7 +33451,7 @@
       </c>
       <c r="K558" t="inlineStr">
         <is>
-          <t>다니엘관203호(小)</t>
+          <t>다니엘관305호(大)</t>
         </is>
       </c>
       <c r="L558" t="inlineStr">
@@ -46439,7 +46447,7 @@
       </c>
       <c r="K772" t="inlineStr">
         <is>
-          <t>다니엘관306호(中)강의실(첨단강의실)</t>
+          <t>사무엘관309호(大)강의실</t>
         </is>
       </c>
       <c r="L772" t="inlineStr">
@@ -46871,7 +46879,11 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I779" t="inlineStr"/>
+      <c r="I779" t="inlineStr">
+        <is>
+          <t>신승원</t>
+        </is>
+      </c>
       <c r="J779" t="inlineStr">
         <is>
           <t>월1~3</t>
@@ -47277,7 +47289,11 @@
           <t>화2~4</t>
         </is>
       </c>
-      <c r="K785" t="inlineStr"/>
+      <c r="K785" t="inlineStr">
+        <is>
+          <t>요한관423호(中)강의실</t>
+        </is>
+      </c>
       <c r="L785" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -49215,7 +49231,7 @@
       </c>
       <c r="K816" t="inlineStr">
         <is>
-          <t>에스라관113호강의실</t>
+          <t>다니엘관305호(大)</t>
         </is>
       </c>
       <c r="L816" t="inlineStr">
@@ -56409,7 +56425,11 @@
           <t>화5~7</t>
         </is>
       </c>
-      <c r="K930" t="inlineStr"/>
+      <c r="K930" t="inlineStr">
+        <is>
+          <t>요한관423호(中)강의실</t>
+        </is>
+      </c>
       <c r="L930" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -60963,7 +60983,7 @@
       </c>
       <c r="K998" t="inlineStr">
         <is>
-          <t>다니엘관305호(大)</t>
+          <t>사무엘관309호(大)강의실</t>
         </is>
       </c>
       <c r="L998" t="inlineStr">
@@ -62657,7 +62677,11 @@
           <t>수5~7</t>
         </is>
       </c>
-      <c r="K1023" t="inlineStr"/>
+      <c r="K1023" t="inlineStr">
+        <is>
+          <t>요한관423호(中)강의실</t>
+        </is>
+      </c>
       <c r="L1023" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -62721,7 +62745,11 @@
           <t>수2~4</t>
         </is>
       </c>
-      <c r="K1024" t="inlineStr"/>
+      <c r="K1024" t="inlineStr">
+        <is>
+          <t>요한관423호(中)강의실</t>
+        </is>
+      </c>
       <c r="L1024" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -67113,7 +67141,11 @@
           <t>월2~4</t>
         </is>
       </c>
-      <c r="K1089" t="inlineStr"/>
+      <c r="K1089" t="inlineStr">
+        <is>
+          <t>요한관423호(中)강의실</t>
+        </is>
+      </c>
       <c r="L1089" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -73169,7 +73201,11 @@
           <t>목6~8</t>
         </is>
       </c>
-      <c r="K1189" t="inlineStr"/>
+      <c r="K1189" t="inlineStr">
+        <is>
+          <t>요한관423호(中)강의실</t>
+        </is>
+      </c>
       <c r="L1189" t="inlineStr">
         <is>
           <t>창의융합대학</t>
@@ -74522,7 +74558,7 @@
       </c>
       <c r="J1211" t="inlineStr">
         <is>
-          <t>목1~3</t>
+          <t>목2~4</t>
         </is>
       </c>
       <c r="K1211" t="inlineStr">
@@ -74582,7 +74618,7 @@
       </c>
       <c r="J1212" t="inlineStr">
         <is>
-          <t>목4~6</t>
+          <t>목5~7</t>
         </is>
       </c>
       <c r="K1212" t="inlineStr">
@@ -77146,7 +77182,7 @@
       </c>
       <c r="J1255" t="inlineStr">
         <is>
-          <t>금5~7</t>
+          <t>목5~7</t>
         </is>
       </c>
       <c r="K1255" t="inlineStr">

</xml_diff>